<commit_message>
fix(ui): harmonize modal colors, improve animations, and update Coretax Agent watchdog security
</commit_message>
<xml_diff>
--- a/Template Impor Dividen - Coretax Agent.xlsx
+++ b/Template Impor Dividen - Coretax Agent.xlsx
@@ -1,35 +1,46 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="76" documentId="11_0B7EEA54247987F80ECAE95015C6D0401322CDF4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CAF08E6E-53D3-50F1-9B1F-A7B2DCCAF143}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Petunjuk" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Referensi" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Info Umum" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Dividen" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Investasi" state="visible" r:id="rId8"/>
+    <sheet name="Petunjuk" sheetId="1" r:id="rId1"/>
+    <sheet name="Referensi" sheetId="2" r:id="rId2"/>
+    <sheet name="Info Umum" sheetId="3" r:id="rId3"/>
+    <sheet name="Dividen" sheetId="4" r:id="rId4"/>
+    <sheet name="Investasi" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
+    <definedName name="ListBentuk">Referensi!$D$2:$D$123</definedName>
     <definedName name="ListJenis">Referensi!$A$2:$A$6</definedName>
+    <definedName name="ListKota">Referensi!$E$2:$E$515</definedName>
     <definedName name="ListKurs">Referensi!$B$2:$B$112</definedName>
     <definedName name="ListTahun">Referensi!$C$2:$C$10</definedName>
-    <definedName name="ListBentuk">Referensi!$D$2:$D$123</definedName>
-    <definedName name="ListKota">Referensi!$E$2:$E$515</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
-<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="A3" authorId="0">
+    <comment ref="A3" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
       <text>
         <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
           <t>WAJIB. Kota/Kabupaten tempat laporan dibuat - tombol "Simpan" di Coretax tetap non-aktif kalau ini kosong.</t>
         </r>
       </text>
@@ -38,15 +49,22 @@
 </comments>
 </file>
 
-<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="A2" authorId="0">
+    <comment ref="A2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0300-000001000000}">
       <text>
         <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
           <t>Baris contoh - boleh dihapus.</t>
         </r>
       </text>
@@ -55,15 +73,22 @@
 </comments>
 </file>
 
-<file path=xl/comments5.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Author</author>
   </authors>
   <commentList>
-    <comment ref="A2" authorId="0">
+    <comment ref="A2" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0400-000001000000}">
       <text>
         <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
           <t>Baris contoh - boleh dihapus.</t>
         </r>
       </text>
@@ -2448,14 +2473,14 @@
     <t>Nilai di atas berlaku untuk SATU laporan (bukan per-baris). Baris dividen &amp; investasi diisi di sheet masing-masing.</t>
   </si>
   <si>
-    <t xml:space="preserve">Pelaporan Ke-
+    <t>Pelaporan Ke-
 (1/2/3)</t>
   </si>
   <si>
     <t>Pemberi Penghasilan</t>
   </si>
   <si>
-    <t xml:space="preserve">Tanggal Diterima
+    <t>Tanggal Diterima
 (YYYY-MM-DD)</t>
   </si>
   <si>
@@ -2471,15 +2496,15 @@
     <t>Nominal Dividen Diinvestasikan</t>
   </si>
   <si>
-    <t xml:space="preserve">Laba Setelah Pajak (Kurs)
+    <t>Laba Setelah Pajak (Kurs)
 [LN saja]</t>
   </si>
   <si>
-    <t xml:space="preserve">Laba Setelah Pajak (Nominal)
+    <t>Laba Setelah Pajak (Nominal)
 [LN saja]</t>
   </si>
   <si>
-    <t xml:space="preserve">Proporsi Kepemilikan Saham (%)
+    <t>Proporsi Kepemilikan Saham (%)
 [LN saja]</t>
   </si>
   <si>
@@ -2489,7 +2514,7 @@
     <t>2024-12-23</t>
   </si>
   <si>
-    <t xml:space="preserve">Tanggal Investasi
+    <t>Tanggal Investasi
 (YYYY-MM-DD)</t>
   </si>
   <si>
@@ -2505,34 +2530,41 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF1B3A6B"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF1B3A6B"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
-    </font>
-    <font>
-      <b/>
+      <name val="Calibri"/>
     </font>
     <font>
       <i/>
+      <sz val="11"/>
       <color rgb="FF888888"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="3">
@@ -2557,10 +2589,18 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -2914,18 +2954,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FF1B3A6B"/>
   </sheetPr>
   <dimension ref="A1:B24"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2941,7 +2981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -2997,7 +3037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -3119,17 +3159,17 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <tabColor rgb="FF2E7D32"/>
   </sheetPr>
   <dimension ref="A1:E515"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="55" customWidth="1"/>
     <col min="2" max="2" width="40" customWidth="1"/>
@@ -3138,7 +3178,7 @@
     <col min="5" max="5" width="45" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>20</v>
       </c>
@@ -3362,7 +3402,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>84</v>
       </c>
@@ -3373,7 +3413,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>87</v>
       </c>
@@ -3384,7 +3424,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>90</v>
       </c>
@@ -3395,7 +3435,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>93</v>
       </c>
@@ -3406,7 +3446,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>96</v>
       </c>
@@ -3417,7 +3457,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>99</v>
       </c>
@@ -3428,7 +3468,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>102</v>
       </c>
@@ -3439,7 +3479,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>105</v>
       </c>
@@ -3450,7 +3490,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>108</v>
       </c>
@@ -3461,7 +3501,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>111</v>
       </c>
@@ -3472,7 +3512,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>114</v>
       </c>
@@ -3483,7 +3523,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>117</v>
       </c>
@@ -3494,7 +3534,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>120</v>
       </c>
@@ -3505,7 +3545,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>123</v>
       </c>
@@ -3516,7 +3556,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>126</v>
       </c>
@@ -3527,7 +3567,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
         <v>129</v>
       </c>
@@ -3538,7 +3578,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B33" t="s">
         <v>132</v>
       </c>
@@ -3549,7 +3589,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B34" t="s">
         <v>135</v>
       </c>
@@ -3560,7 +3600,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B35" t="s">
         <v>138</v>
       </c>
@@ -3571,7 +3611,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B36" t="s">
         <v>141</v>
       </c>
@@ -3582,7 +3622,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
         <v>144</v>
       </c>
@@ -3593,7 +3633,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>147</v>
       </c>
@@ -3604,7 +3644,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
         <v>150</v>
       </c>
@@ -3615,7 +3655,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
         <v>153</v>
       </c>
@@ -3626,7 +3666,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>156</v>
       </c>
@@ -3637,7 +3677,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
         <v>159</v>
       </c>
@@ -3648,7 +3688,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
         <v>162</v>
       </c>
@@ -3659,7 +3699,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
         <v>165</v>
       </c>
@@ -3670,7 +3710,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
         <v>168</v>
       </c>
@@ -3681,7 +3721,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
         <v>171</v>
       </c>
@@ -3692,7 +3732,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
         <v>174</v>
       </c>
@@ -3703,7 +3743,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
         <v>177</v>
       </c>
@@ -3714,7 +3754,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
         <v>180</v>
       </c>
@@ -3725,7 +3765,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
         <v>183</v>
       </c>
@@ -3736,7 +3776,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
         <v>186</v>
       </c>
@@ -3747,7 +3787,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
         <v>189</v>
       </c>
@@ -3758,7 +3798,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
         <v>192</v>
       </c>
@@ -3769,7 +3809,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
         <v>195</v>
       </c>
@@ -3780,7 +3820,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
         <v>198</v>
       </c>
@@ -3791,7 +3831,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
         <v>201</v>
       </c>
@@ -3802,7 +3842,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B57" t="s">
         <v>204</v>
       </c>
@@ -3813,7 +3853,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B58" t="s">
         <v>207</v>
       </c>
@@ -3824,7 +3864,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B59" t="s">
         <v>210</v>
       </c>
@@ -3835,7 +3875,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B60" t="s">
         <v>213</v>
       </c>
@@ -3846,7 +3886,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B61" t="s">
         <v>216</v>
       </c>
@@ -3857,7 +3897,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
         <v>219</v>
       </c>
@@ -3868,7 +3908,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
         <v>222</v>
       </c>
@@ -3879,7 +3919,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
         <v>225</v>
       </c>
@@ -3890,7 +3930,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B65" t="s">
         <v>228</v>
       </c>
@@ -3901,7 +3941,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B66" t="s">
         <v>231</v>
       </c>
@@ -3912,7 +3952,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
         <v>234</v>
       </c>
@@ -3923,7 +3963,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B68" t="s">
         <v>237</v>
       </c>
@@ -3934,7 +3974,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B69" t="s">
         <v>240</v>
       </c>
@@ -3945,7 +3985,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B70" t="s">
         <v>243</v>
       </c>
@@ -3956,7 +3996,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B71" t="s">
         <v>246</v>
       </c>
@@ -3967,7 +4007,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B72" t="s">
         <v>249</v>
       </c>
@@ -3978,7 +4018,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B73" t="s">
         <v>252</v>
       </c>
@@ -3989,7 +4029,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B74" t="s">
         <v>255</v>
       </c>
@@ -4000,7 +4040,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B75" t="s">
         <v>258</v>
       </c>
@@ -4011,7 +4051,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B76" t="s">
         <v>261</v>
       </c>
@@ -4022,7 +4062,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B77" t="s">
         <v>264</v>
       </c>
@@ -4033,7 +4073,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B78" t="s">
         <v>267</v>
       </c>
@@ -4044,7 +4084,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B79" t="s">
         <v>270</v>
       </c>
@@ -4055,7 +4095,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B80" t="s">
         <v>273</v>
       </c>
@@ -4066,7 +4106,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B81" t="s">
         <v>276</v>
       </c>
@@ -4077,7 +4117,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B82" t="s">
         <v>279</v>
       </c>
@@ -4088,7 +4128,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B83" t="s">
         <v>282</v>
       </c>
@@ -4099,7 +4139,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B84" t="s">
         <v>285</v>
       </c>
@@ -4110,7 +4150,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B85" t="s">
         <v>288</v>
       </c>
@@ -4121,7 +4161,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B86" t="s">
         <v>291</v>
       </c>
@@ -4132,7 +4172,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B87" t="s">
         <v>294</v>
       </c>
@@ -4143,7 +4183,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B88" t="s">
         <v>297</v>
       </c>
@@ -4154,7 +4194,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B89" t="s">
         <v>300</v>
       </c>
@@ -4165,7 +4205,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B90" t="s">
         <v>303</v>
       </c>
@@ -4176,7 +4216,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B91" t="s">
         <v>306</v>
       </c>
@@ -4187,7 +4227,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B92" t="s">
         <v>309</v>
       </c>
@@ -4198,7 +4238,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B93" t="s">
         <v>312</v>
       </c>
@@ -4209,7 +4249,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B94" t="s">
         <v>315</v>
       </c>
@@ -4220,7 +4260,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B95" t="s">
         <v>318</v>
       </c>
@@ -4231,7 +4271,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B96" t="s">
         <v>321</v>
       </c>
@@ -4242,7 +4282,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B97" t="s">
         <v>324</v>
       </c>
@@ -4253,7 +4293,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B98" t="s">
         <v>327</v>
       </c>
@@ -4264,7 +4304,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B99" t="s">
         <v>330</v>
       </c>
@@ -4275,7 +4315,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B100" t="s">
         <v>333</v>
       </c>
@@ -4286,7 +4326,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B101" t="s">
         <v>336</v>
       </c>
@@ -4297,7 +4337,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B102" t="s">
         <v>339</v>
       </c>
@@ -4308,7 +4348,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B103" t="s">
         <v>342</v>
       </c>
@@ -4319,7 +4359,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B104" t="s">
         <v>345</v>
       </c>
@@ -4330,7 +4370,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B105" t="s">
         <v>348</v>
       </c>
@@ -4341,7 +4381,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B106" t="s">
         <v>351</v>
       </c>
@@ -4352,7 +4392,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B107" t="s">
         <v>354</v>
       </c>
@@ -4363,7 +4403,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B108" t="s">
         <v>357</v>
       </c>
@@ -4374,7 +4414,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B109" t="s">
         <v>360</v>
       </c>
@@ -4385,7 +4425,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B110" t="s">
         <v>363</v>
       </c>
@@ -4396,7 +4436,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B111" t="s">
         <v>366</v>
       </c>
@@ -4407,7 +4447,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B112" t="s">
         <v>369</v>
       </c>
@@ -4418,7 +4458,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D113" t="s">
         <v>372</v>
       </c>
@@ -4426,7 +4466,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D114" t="s">
         <v>374</v>
       </c>
@@ -4434,7 +4474,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D115" t="s">
         <v>376</v>
       </c>
@@ -4442,7 +4482,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D116" t="s">
         <v>378</v>
       </c>
@@ -4450,7 +4490,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D117" t="s">
         <v>380</v>
       </c>
@@ -4458,7 +4498,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D118" t="s">
         <v>382</v>
       </c>
@@ -4466,7 +4506,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D119" t="s">
         <v>384</v>
       </c>
@@ -4474,7 +4514,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D120" t="s">
         <v>386</v>
       </c>
@@ -4482,7 +4522,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D121" t="s">
         <v>388</v>
       </c>
@@ -4490,7 +4530,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D122" t="s">
         <v>390</v>
       </c>
@@ -4498,7 +4538,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D123" t="s">
         <v>392</v>
       </c>
@@ -4506,1985 +4546,1985 @@
         <v>393</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E124" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E125" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E126" t="s">
         <v>396</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E127" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="4:5" x14ac:dyDescent="0.25">
       <c r="E128" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E129" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E130" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E131" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E132" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E133" t="s">
         <v>403</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E134" t="s">
         <v>404</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E135" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E136" t="s">
         <v>406</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E137" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E138" t="s">
         <v>408</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E139" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E140" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E141" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E142" t="s">
         <v>412</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E143" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E144" t="s">
         <v>414</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E145" t="s">
         <v>415</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E146" t="s">
         <v>416</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E147" t="s">
         <v>417</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E148" t="s">
         <v>418</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E149" t="s">
         <v>419</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E150" t="s">
         <v>420</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E151" t="s">
         <v>421</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E152" t="s">
         <v>422</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E153" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E154" t="s">
         <v>424</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E155" t="s">
         <v>425</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E156" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E157" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E158" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E159" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E160" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E161" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E162" t="s">
         <v>432</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E163" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E164" t="s">
         <v>434</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E165" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E166" t="s">
         <v>436</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E167" t="s">
         <v>437</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E168" t="s">
         <v>438</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E169" t="s">
         <v>439</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E170" t="s">
         <v>440</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E171" t="s">
         <v>441</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E172" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E173" t="s">
         <v>443</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E174" t="s">
         <v>444</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E175" t="s">
         <v>445</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E176" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E177" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E178" t="s">
         <v>448</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E179" t="s">
         <v>449</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E180" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E181" t="s">
         <v>451</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E182" t="s">
         <v>452</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E183" t="s">
         <v>453</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E184" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E185" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E186" t="s">
         <v>456</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E187" t="s">
         <v>457</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E188" t="s">
         <v>458</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E189" t="s">
         <v>459</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E190" t="s">
         <v>460</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E191" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E192" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E193" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E194" t="s">
         <v>464</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E195" t="s">
         <v>465</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E196" t="s">
         <v>466</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E197" t="s">
         <v>467</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E198" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E199" t="s">
         <v>469</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E200" t="s">
         <v>470</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E201" t="s">
         <v>471</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E202" t="s">
         <v>472</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E203" t="s">
         <v>473</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E204" t="s">
         <v>474</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E205" t="s">
         <v>475</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E206" t="s">
         <v>476</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E207" t="s">
         <v>477</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E208" t="s">
         <v>478</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E209" t="s">
         <v>479</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E210" t="s">
         <v>480</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E211" t="s">
         <v>481</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E212" t="s">
         <v>482</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E213" t="s">
         <v>483</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E214" t="s">
         <v>484</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E215" t="s">
         <v>485</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E216" t="s">
         <v>486</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E217" t="s">
         <v>487</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E218" t="s">
         <v>488</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E219" t="s">
         <v>489</v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="220" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E220" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="221" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E221" t="s">
         <v>491</v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="222" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E222" t="s">
         <v>492</v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="223" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E223" t="s">
         <v>493</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="224" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E224" t="s">
         <v>494</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="225" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E225" t="s">
         <v>495</v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="226" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E226" t="s">
         <v>496</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E227" t="s">
         <v>497</v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="228" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E228" t="s">
         <v>498</v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="229" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E229" t="s">
         <v>499</v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="230" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E230" t="s">
         <v>500</v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="231" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E231" t="s">
         <v>501</v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="232" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E232" t="s">
         <v>502</v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E233" t="s">
         <v>503</v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="234" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E234" t="s">
         <v>504</v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="235" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E235" t="s">
         <v>505</v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="236" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E236" t="s">
         <v>506</v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="237" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E237" t="s">
         <v>507</v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="238" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E238" t="s">
         <v>508</v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="239" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E239" t="s">
         <v>509</v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="240" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E240" t="s">
         <v>510</v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="241" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E241" t="s">
         <v>511</v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="242" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E242" t="s">
         <v>512</v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="243" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E243" t="s">
         <v>513</v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="244" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E244" t="s">
         <v>514</v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="245" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E245" t="s">
         <v>515</v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="246" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E246" t="s">
         <v>516</v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="247" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E247" t="s">
         <v>517</v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="248" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E248" t="s">
         <v>518</v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="249" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E249" t="s">
         <v>519</v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="250" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E250" t="s">
         <v>520</v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="251" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E251" t="s">
         <v>521</v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="252" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E252" t="s">
         <v>522</v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="253" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E253" t="s">
         <v>523</v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="254" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E254" t="s">
         <v>524</v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="255" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E255" t="s">
         <v>525</v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="256" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E256" t="s">
         <v>526</v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="257" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E257" t="s">
         <v>527</v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="258" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E258" t="s">
         <v>528</v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="259" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E259" t="s">
         <v>529</v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="260" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E260" t="s">
         <v>530</v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="261" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E261" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="262" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E262" t="s">
         <v>532</v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="263" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E263" t="s">
         <v>533</v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="264" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E264" t="s">
         <v>534</v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="265" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E265" t="s">
         <v>535</v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="266" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E266" t="s">
         <v>536</v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="267" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E267" t="s">
         <v>537</v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="268" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E268" t="s">
         <v>538</v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="269" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E269" t="s">
         <v>539</v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="270" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E270" t="s">
         <v>540</v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="271" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E271" t="s">
         <v>541</v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="272" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E272" t="s">
         <v>542</v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="273" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E273" t="s">
         <v>543</v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="274" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E274" t="s">
         <v>544</v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="275" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E275" t="s">
         <v>545</v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="276" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E276" t="s">
         <v>546</v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="277" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E277" t="s">
         <v>547</v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="278" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E278" t="s">
         <v>548</v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="279" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E279" t="s">
         <v>549</v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="280" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E280" t="s">
         <v>550</v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="281" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E281" t="s">
         <v>551</v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="282" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E282" t="s">
         <v>552</v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="283" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E283" t="s">
         <v>553</v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="284" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E284" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="285" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E285" t="s">
         <v>555</v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="286" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E286" t="s">
         <v>556</v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="287" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E287" t="s">
         <v>557</v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="288" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E288" t="s">
         <v>558</v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="289" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E289" t="s">
         <v>559</v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="290" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E290" t="s">
         <v>560</v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="291" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E291" t="s">
         <v>561</v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="292" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E292" t="s">
         <v>562</v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="293" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E293" t="s">
         <v>563</v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="294" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E294" t="s">
         <v>564</v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="295" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E295" t="s">
         <v>565</v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="296" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E296" t="s">
         <v>566</v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="297" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E297" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="298" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E298" t="s">
         <v>568</v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="299" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E299" t="s">
         <v>569</v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="300" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E300" t="s">
         <v>570</v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="301" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E301" t="s">
         <v>571</v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="302" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E302" t="s">
         <v>572</v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="303" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E303" t="s">
         <v>573</v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="304" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E304" t="s">
         <v>574</v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="305" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E305" t="s">
         <v>575</v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="306" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E306" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="307" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E307" t="s">
         <v>577</v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="308" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E308" t="s">
         <v>578</v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="309" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E309" t="s">
         <v>579</v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="310" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E310" t="s">
         <v>580</v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="311" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E311" t="s">
         <v>581</v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="312" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E312" t="s">
         <v>582</v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="313" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E313" t="s">
         <v>583</v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="314" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E314" t="s">
         <v>584</v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="315" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E315" t="s">
         <v>585</v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="316" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E316" t="s">
         <v>586</v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="317" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E317" t="s">
         <v>587</v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="318" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E318" t="s">
         <v>588</v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="319" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E319" t="s">
         <v>589</v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="320" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E320" t="s">
         <v>590</v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="321" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E321" t="s">
         <v>591</v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="322" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E322" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="323" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E323" t="s">
         <v>593</v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="324" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E324" t="s">
         <v>594</v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="325" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E325" t="s">
         <v>595</v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="326" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E326" t="s">
         <v>596</v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="327" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E327" t="s">
         <v>597</v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="328" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E328" t="s">
         <v>598</v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="329" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E329" t="s">
         <v>599</v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="330" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E330" t="s">
         <v>600</v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="331" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E331" t="s">
         <v>601</v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="332" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E332" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="333" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E333" t="s">
         <v>603</v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="334" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E334" t="s">
         <v>604</v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="335" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E335" t="s">
         <v>605</v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="336" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E336" t="s">
         <v>606</v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="337" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E337" t="s">
         <v>607</v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="338" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E338" t="s">
         <v>608</v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="339" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E339" t="s">
         <v>609</v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="340" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E340" t="s">
         <v>610</v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="341" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E341" t="s">
         <v>611</v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="342" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E342" t="s">
         <v>612</v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="343" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E343" t="s">
         <v>613</v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="344" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E344" t="s">
         <v>614</v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="345" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E345" t="s">
         <v>615</v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="346" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E346" t="s">
         <v>616</v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="347" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E347" t="s">
         <v>617</v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="348" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E348" t="s">
         <v>618</v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="349" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E349" t="s">
         <v>619</v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="350" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E350" t="s">
         <v>620</v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="351" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E351" t="s">
         <v>621</v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="352" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E352" t="s">
         <v>622</v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="353" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E353" t="s">
         <v>623</v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="354" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E354" t="s">
         <v>624</v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="355" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E355" t="s">
         <v>625</v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="356" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E356" t="s">
         <v>626</v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="357" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E357" t="s">
         <v>627</v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="358" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E358" t="s">
         <v>628</v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="359" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E359" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="360" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E360" t="s">
         <v>630</v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="361" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E361" t="s">
         <v>631</v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="362" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E362" t="s">
         <v>632</v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="363" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E363" t="s">
         <v>633</v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="364" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E364" t="s">
         <v>634</v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="365" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E365" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="366" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E366" t="s">
         <v>636</v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="367" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E367" t="s">
         <v>637</v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="368" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E368" t="s">
         <v>638</v>
       </c>
     </row>
-    <row r="369" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="369" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E369" t="s">
         <v>639</v>
       </c>
     </row>
-    <row r="370" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="370" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E370" t="s">
         <v>640</v>
       </c>
     </row>
-    <row r="371" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="371" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E371" t="s">
         <v>641</v>
       </c>
     </row>
-    <row r="372" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="372" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E372" t="s">
         <v>642</v>
       </c>
     </row>
-    <row r="373" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="373" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E373" t="s">
         <v>643</v>
       </c>
     </row>
-    <row r="374" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="374" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E374" t="s">
         <v>644</v>
       </c>
     </row>
-    <row r="375" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="375" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E375" t="s">
         <v>645</v>
       </c>
     </row>
-    <row r="376" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="376" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E376" t="s">
         <v>646</v>
       </c>
     </row>
-    <row r="377" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="377" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E377" t="s">
         <v>647</v>
       </c>
     </row>
-    <row r="378" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="378" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E378" t="s">
         <v>648</v>
       </c>
     </row>
-    <row r="379" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="379" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E379" t="s">
         <v>649</v>
       </c>
     </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="380" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E380" t="s">
         <v>650</v>
       </c>
     </row>
-    <row r="381" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="381" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E381" t="s">
         <v>651</v>
       </c>
     </row>
-    <row r="382" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="382" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E382" t="s">
         <v>652</v>
       </c>
     </row>
-    <row r="383" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="383" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E383" t="s">
         <v>653</v>
       </c>
     </row>
-    <row r="384" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="384" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E384" t="s">
         <v>654</v>
       </c>
     </row>
-    <row r="385" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="385" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E385" t="s">
         <v>655</v>
       </c>
     </row>
-    <row r="386" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="386" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E386" t="s">
         <v>656</v>
       </c>
     </row>
-    <row r="387" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="387" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E387" t="s">
         <v>657</v>
       </c>
     </row>
-    <row r="388" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="388" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E388" t="s">
         <v>658</v>
       </c>
     </row>
-    <row r="389" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="389" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E389" t="s">
         <v>659</v>
       </c>
     </row>
-    <row r="390" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="390" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E390" t="s">
         <v>660</v>
       </c>
     </row>
-    <row r="391" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="391" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E391" t="s">
         <v>661</v>
       </c>
     </row>
-    <row r="392" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="392" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E392" t="s">
         <v>662</v>
       </c>
     </row>
-    <row r="393" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="393" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E393" t="s">
         <v>663</v>
       </c>
     </row>
-    <row r="394" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="394" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E394" t="s">
         <v>664</v>
       </c>
     </row>
-    <row r="395" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="395" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E395" t="s">
         <v>665</v>
       </c>
     </row>
-    <row r="396" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="396" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E396" t="s">
         <v>666</v>
       </c>
     </row>
-    <row r="397" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="397" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E397" t="s">
         <v>667</v>
       </c>
     </row>
-    <row r="398" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="398" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E398" t="s">
         <v>668</v>
       </c>
     </row>
-    <row r="399" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="399" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E399" t="s">
         <v>669</v>
       </c>
     </row>
-    <row r="400" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="400" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E400" t="s">
         <v>670</v>
       </c>
     </row>
-    <row r="401" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="401" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E401" t="s">
         <v>671</v>
       </c>
     </row>
-    <row r="402" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="402" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E402" t="s">
         <v>672</v>
       </c>
     </row>
-    <row r="403" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="403" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E403" t="s">
         <v>673</v>
       </c>
     </row>
-    <row r="404" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="404" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E404" t="s">
         <v>674</v>
       </c>
     </row>
-    <row r="405" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="405" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E405" t="s">
         <v>675</v>
       </c>
     </row>
-    <row r="406" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="406" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E406" t="s">
         <v>676</v>
       </c>
     </row>
-    <row r="407" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="407" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E407" t="s">
         <v>677</v>
       </c>
     </row>
-    <row r="408" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="408" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E408" t="s">
         <v>678</v>
       </c>
     </row>
-    <row r="409" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="409" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E409" t="s">
         <v>679</v>
       </c>
     </row>
-    <row r="410" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="410" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E410" t="s">
         <v>680</v>
       </c>
     </row>
-    <row r="411" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="411" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E411" t="s">
         <v>681</v>
       </c>
     </row>
-    <row r="412" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="412" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E412" t="s">
         <v>682</v>
       </c>
     </row>
-    <row r="413" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="413" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E413" t="s">
         <v>683</v>
       </c>
     </row>
-    <row r="414" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="414" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E414" t="s">
         <v>684</v>
       </c>
     </row>
-    <row r="415" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="415" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E415" t="s">
         <v>685</v>
       </c>
     </row>
-    <row r="416" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="416" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E416" t="s">
         <v>686</v>
       </c>
     </row>
-    <row r="417" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="417" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E417" t="s">
         <v>687</v>
       </c>
     </row>
-    <row r="418" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="418" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E418" t="s">
         <v>688</v>
       </c>
     </row>
-    <row r="419" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="419" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E419" t="s">
         <v>689</v>
       </c>
     </row>
-    <row r="420" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="420" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E420" t="s">
         <v>690</v>
       </c>
     </row>
-    <row r="421" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="421" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E421" t="s">
         <v>691</v>
       </c>
     </row>
-    <row r="422" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="422" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E422" t="s">
         <v>692</v>
       </c>
     </row>
-    <row r="423" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="423" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E423" t="s">
         <v>693</v>
       </c>
     </row>
-    <row r="424" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="424" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E424" t="s">
         <v>694</v>
       </c>
     </row>
-    <row r="425" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="425" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E425" t="s">
         <v>695</v>
       </c>
     </row>
-    <row r="426" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="426" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E426" t="s">
         <v>696</v>
       </c>
     </row>
-    <row r="427" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="427" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E427" t="s">
         <v>697</v>
       </c>
     </row>
-    <row r="428" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="428" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E428" t="s">
         <v>698</v>
       </c>
     </row>
-    <row r="429" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="429" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E429" t="s">
         <v>699</v>
       </c>
     </row>
-    <row r="430" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="430" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E430" t="s">
         <v>700</v>
       </c>
     </row>
-    <row r="431" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="431" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E431" t="s">
         <v>701</v>
       </c>
     </row>
-    <row r="432" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="432" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E432" t="s">
         <v>702</v>
       </c>
     </row>
-    <row r="433" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="433" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E433" t="s">
         <v>703</v>
       </c>
     </row>
-    <row r="434" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="434" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E434" t="s">
         <v>704</v>
       </c>
     </row>
-    <row r="435" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="435" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E435" t="s">
         <v>705</v>
       </c>
     </row>
-    <row r="436" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="436" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E436" t="s">
         <v>706</v>
       </c>
     </row>
-    <row r="437" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="437" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E437" t="s">
         <v>707</v>
       </c>
     </row>
-    <row r="438" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="438" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E438" t="s">
         <v>708</v>
       </c>
     </row>
-    <row r="439" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="439" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E439" t="s">
         <v>709</v>
       </c>
     </row>
-    <row r="440" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="440" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E440" t="s">
         <v>710</v>
       </c>
     </row>
-    <row r="441" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="441" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E441" t="s">
         <v>711</v>
       </c>
     </row>
-    <row r="442" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="442" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E442" t="s">
         <v>712</v>
       </c>
     </row>
-    <row r="443" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="443" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E443" t="s">
         <v>713</v>
       </c>
     </row>
-    <row r="444" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="444" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E444" t="s">
         <v>714</v>
       </c>
     </row>
-    <row r="445" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="445" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E445" t="s">
         <v>715</v>
       </c>
     </row>
-    <row r="446" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="446" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E446" t="s">
         <v>716</v>
       </c>
     </row>
-    <row r="447" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="447" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E447" t="s">
         <v>717</v>
       </c>
     </row>
-    <row r="448" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="448" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E448" t="s">
         <v>718</v>
       </c>
     </row>
-    <row r="449" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="449" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E449" t="s">
         <v>719</v>
       </c>
     </row>
-    <row r="450" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="450" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E450" t="s">
         <v>720</v>
       </c>
     </row>
-    <row r="451" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="451" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E451" t="s">
         <v>721</v>
       </c>
     </row>
-    <row r="452" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="452" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E452" t="s">
         <v>722</v>
       </c>
     </row>
-    <row r="453" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="453" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E453" t="s">
         <v>723</v>
       </c>
     </row>
-    <row r="454" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="454" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E454" t="s">
         <v>724</v>
       </c>
     </row>
-    <row r="455" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="455" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E455" t="s">
         <v>725</v>
       </c>
     </row>
-    <row r="456" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="456" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E456" t="s">
         <v>726</v>
       </c>
     </row>
-    <row r="457" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="457" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E457" t="s">
         <v>727</v>
       </c>
     </row>
-    <row r="458" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="458" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E458" t="s">
         <v>728</v>
       </c>
     </row>
-    <row r="459" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="459" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E459" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="460" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="460" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E460" t="s">
         <v>730</v>
       </c>
     </row>
-    <row r="461" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="461" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E461" t="s">
         <v>731</v>
       </c>
     </row>
-    <row r="462" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="462" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E462" t="s">
         <v>732</v>
       </c>
     </row>
-    <row r="463" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="463" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E463" t="s">
         <v>733</v>
       </c>
     </row>
-    <row r="464" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="464" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E464" t="s">
         <v>734</v>
       </c>
     </row>
-    <row r="465" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="465" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E465" t="s">
         <v>735</v>
       </c>
     </row>
-    <row r="466" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="466" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E466" t="s">
         <v>736</v>
       </c>
     </row>
-    <row r="467" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="467" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E467" t="s">
         <v>737</v>
       </c>
     </row>
-    <row r="468" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="468" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E468" t="s">
         <v>738</v>
       </c>
     </row>
-    <row r="469" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="469" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E469" t="s">
         <v>739</v>
       </c>
     </row>
-    <row r="470" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="470" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E470" t="s">
         <v>740</v>
       </c>
     </row>
-    <row r="471" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="471" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E471" t="s">
         <v>741</v>
       </c>
     </row>
-    <row r="472" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="472" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E472" t="s">
         <v>742</v>
       </c>
     </row>
-    <row r="473" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="473" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E473" t="s">
         <v>743</v>
       </c>
     </row>
-    <row r="474" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="474" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E474" t="s">
         <v>744</v>
       </c>
     </row>
-    <row r="475" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="475" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E475" t="s">
         <v>745</v>
       </c>
     </row>
-    <row r="476" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="476" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E476" t="s">
         <v>746</v>
       </c>
     </row>
-    <row r="477" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="477" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E477" t="s">
         <v>747</v>
       </c>
     </row>
-    <row r="478" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="478" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E478" t="s">
         <v>748</v>
       </c>
     </row>
-    <row r="479" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="479" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E479" t="s">
         <v>749</v>
       </c>
     </row>
-    <row r="480" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="480" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E480" t="s">
         <v>750</v>
       </c>
     </row>
-    <row r="481" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="481" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E481" t="s">
         <v>751</v>
       </c>
     </row>
-    <row r="482" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="482" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E482" t="s">
         <v>752</v>
       </c>
     </row>
-    <row r="483" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="483" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E483" t="s">
         <v>753</v>
       </c>
     </row>
-    <row r="484" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="484" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E484" t="s">
         <v>754</v>
       </c>
     </row>
-    <row r="485" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="485" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E485" t="s">
         <v>755</v>
       </c>
     </row>
-    <row r="486" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="486" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E486" t="s">
         <v>756</v>
       </c>
     </row>
-    <row r="487" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="487" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E487" t="s">
         <v>757</v>
       </c>
     </row>
-    <row r="488" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="488" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E488" t="s">
         <v>758</v>
       </c>
     </row>
-    <row r="489" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="489" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E489" t="s">
         <v>759</v>
       </c>
     </row>
-    <row r="490" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="490" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E490" t="s">
         <v>760</v>
       </c>
     </row>
-    <row r="491" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="491" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E491" t="s">
         <v>761</v>
       </c>
     </row>
-    <row r="492" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="492" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E492" t="s">
         <v>762</v>
       </c>
     </row>
-    <row r="493" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="493" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E493" t="s">
         <v>763</v>
       </c>
     </row>
-    <row r="494" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="494" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E494" t="s">
         <v>764</v>
       </c>
     </row>
-    <row r="495" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="495" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E495" t="s">
         <v>765</v>
       </c>
     </row>
-    <row r="496" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="496" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E496" t="s">
         <v>766</v>
       </c>
     </row>
-    <row r="497" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="497" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E497" t="s">
         <v>767</v>
       </c>
     </row>
-    <row r="498" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="498" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E498" t="s">
         <v>768</v>
       </c>
     </row>
-    <row r="499" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="499" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E499" t="s">
         <v>769</v>
       </c>
     </row>
-    <row r="500" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="500" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E500" t="s">
         <v>770</v>
       </c>
     </row>
-    <row r="501" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="501" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E501" t="s">
         <v>771</v>
       </c>
     </row>
-    <row r="502" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="502" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E502" t="s">
         <v>772</v>
       </c>
     </row>
-    <row r="503" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="503" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E503" t="s">
         <v>773</v>
       </c>
     </row>
-    <row r="504" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="504" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E504" t="s">
         <v>774</v>
       </c>
     </row>
-    <row r="505" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="505" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E505" t="s">
         <v>775</v>
       </c>
     </row>
-    <row r="506" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="506" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E506" t="s">
         <v>776</v>
       </c>
     </row>
-    <row r="507" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="507" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E507" t="s">
         <v>777</v>
       </c>
     </row>
-    <row r="508" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="508" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E508" t="s">
         <v>778</v>
       </c>
     </row>
-    <row r="509" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="509" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E509" t="s">
         <v>779</v>
       </c>
     </row>
-    <row r="510" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="510" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E510" t="s">
         <v>780</v>
       </c>
     </row>
-    <row r="511" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="511" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E511" t="s">
         <v>781</v>
       </c>
     </row>
-    <row r="512" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="512" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E512" t="s">
         <v>782</v>
       </c>
     </row>
-    <row r="513" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="513" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E513" t="s">
         <v>783</v>
       </c>
     </row>
-    <row r="514" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="514" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E514" t="s">
         <v>784</v>
       </c>
     </row>
-    <row r="515" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="515" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E515" t="s">
         <v>785</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor rgb="FF1B3A6B"/>
   </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>786</v>
       </c>
@@ -6513,23 +6553,23 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" showErrorMessage="1" errorStyle="stop" errorTitle="Kota tidak valid" error="Pilih Kota/Kabupaten dari daftar (lihat sheet Referensi)." sqref="B3">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Kota tidak valid" error="Pilih Kota/Kabupaten dari daftar (lihat sheet Referensi)." sqref="B3" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>ListKota</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <tabColor rgb="FFF9A825"/>
   </sheetPr>
-  <dimension ref="A1:L201"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <dimension ref="A1:L2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -6544,7 +6584,7 @@
     <col min="12" max="12" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>791</v>
       </c>
@@ -6610,289 +6650,43 @@
       <c r="I2" s="5">
         <v>100000000</v>
       </c>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="182" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="183" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="185" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="186" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="193" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="195" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="197" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="198" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="199" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.25"/>
-    <row r="201" spans="1:12" x14ac:dyDescent="0.25"/>
+    </row>
   </sheetData>
-  <dataValidations count="20">
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Angka tidak valid" error="Isi bilangan bulat antara 1 dan 3. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="A10:A201">
+  <dataValidations count="6">
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Angka tidak valid" error="Isi bilangan bulat antara 1 dan 3. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="A2:A201" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>1</formula1>
       <formula2>3</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Angka tidak valid" error="Isi bilangan bulat antara 1 dan 3. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="A2:A201">
-      <formula1>1</formula1>
-      <formula2>3</formula2>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="B10:B201">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="B2:B201" xr:uid="{00000000-0002-0000-0300-000002000000}">
       <formula1>ListTahun</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="B2:B201">
-      <formula1>ListTahun</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="C10:C201">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="C2:C201" xr:uid="{00000000-0002-0000-0300-000004000000}">
       <formula1>ListJenis</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="C2:C201">
-      <formula1>ListJenis</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="F10:F201">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="J2:J201 H2:H201 F2:F201" xr:uid="{00000000-0002-0000-0300-000006000000}">
       <formula1>ListKurs</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="F2:F201">
-      <formula1>ListKurs</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Angka tidak valid" error="Isi angka minimal 1. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="G10:G201">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Angka tidak valid" error="Isi angka minimal 1. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="K2:K201 I2:I201 G2:G201" xr:uid="{00000000-0002-0000-0300-000008000000}">
       <formula1>1</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Angka tidak valid" error="Isi angka minimal 1. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="G2:G201">
-      <formula1>1</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="H10:H201">
-      <formula1>ListKurs</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="H2:H201">
-      <formula1>ListKurs</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Angka tidak valid" error="Isi angka minimal 1. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="I10:I201">
-      <formula1>1</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Angka tidak valid" error="Isi angka minimal 1. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="I2:I201">
-      <formula1>1</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="J10:J201">
-      <formula1>ListKurs</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="J2:J201">
-      <formula1>ListKurs</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Angka tidak valid" error="Isi angka minimal 1. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="K10:K201">
-      <formula1>1</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Angka tidak valid" error="Isi angka minimal 1. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="K2:K201">
-      <formula1>1</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Angka tidak valid" error="Isi angka antara 0 dan 100. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="L10:L201">
-      <formula1>0</formula1>
-      <formula2>100</formula2>
-    </dataValidation>
-    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Angka tidak valid" error="Isi angka antara 0 dan 100. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="L2:L201">
+    <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Angka tidak valid" error="Isi angka antara 0 dan 100. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="L2:L201" xr:uid="{00000000-0002-0000-0300-000012000000}">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <tabColor rgb="FFF9A825"/>
   </sheetPr>
-  <dimension ref="A1:F201"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
@@ -6902,7 +6696,7 @@
     <col min="6" max="6" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>791</v>
       </c>
@@ -6942,242 +6736,27 @@
         <v>100000000</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="190" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.25"/>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <dataValidations count="10">
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Angka tidak valid" error="Isi bilangan bulat antara 1 dan 3. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="A10:A201">
+  <dataValidations count="5">
+    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorTitle="Angka tidak valid" error="Isi bilangan bulat antara 1 dan 3. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="A2:A201" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>1</formula1>
       <formula2>3</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Angka tidak valid" error="Isi bilangan bulat antara 1 dan 3. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="A2:A201">
-      <formula1>1</formula1>
-      <formula2>3</formula2>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="B10:B201">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="B2:B201" xr:uid="{00000000-0002-0000-0400-000002000000}">
       <formula1>ListTahun</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="B2:B201">
-      <formula1>ListTahun</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="D10:D201">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="D2:D201" xr:uid="{00000000-0002-0000-0400-000004000000}">
       <formula1>ListBentuk</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="D2:D201">
-      <formula1>ListBentuk</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="E10:E201">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="E2:E201" xr:uid="{00000000-0002-0000-0400-000006000000}">
       <formula1>ListKurs</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Nilai tidak valid" error="Pilih salah satu nilai dari daftar (lihat sheet Referensi)." sqref="E2:E201">
-      <formula1>ListKurs</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Angka tidak valid" error="Isi angka minimal 1. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="F10:F201">
-      <formula1>1</formula1>
-    </dataValidation>
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Angka tidak valid" error="Isi angka minimal 1. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="F2:F201">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="Angka tidak valid" error="Isi angka minimal 1. Jangan pakai pemisah ribuan (titik/koma); desimal boleh pakai koma/titik sesuai Excel Anda." sqref="F2:F201" xr:uid="{00000000-0002-0000-0400-000008000000}">
       <formula1>1</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>